<commit_message>
Add Excel-driven patient vital signs
</commit_message>
<xml_diff>
--- a/outputs/russicaptor-template/Exercise_Demo.xlsx
+++ b/outputs/russicaptor-template/Exercise_Demo.xlsx
@@ -2,18 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R0251d0b713ca492b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patients" sheetId="2" r:id="R131cac14d2144fcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Locations" sheetId="3" r:id="Ra7306a26e3844f12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InterventionOptions" sheetId="4" r:id="R50c689d75d0541c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interventions" sheetId="5" r:id="R5af730f47a794179"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MedicationOptions" sheetId="6" r:id="R8ebd97e94804482e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MedicationAdministrations" sheetId="7" r:id="Rdf6ff3e24ea54e88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="8" r:id="R6cc5d831e9b54eb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labs" sheetId="9" r:id="R73ecbf3af6f34a55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imaging" sheetId="10" r:id="Ra4698eb9c6f2400e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="11" r:id="R1099ba9104c2495f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="12" r:id="R4f5742e301bf4ec4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R8daf2a56868f4873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patients" sheetId="2" r:id="R61742e71a9484d88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Locations" sheetId="3" r:id="R0f30f8bbbfce4a47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InterventionOptions" sheetId="4" r:id="R86d6444d6c174279"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interventions" sheetId="5" r:id="R64ece465235845ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MedicationOptions" sheetId="6" r:id="Rd3feae92d421400a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MedicationAdministrations" sheetId="7" r:id="Ra667402d458b4935"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="8" r:id="R6f5da5671dad4516"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labs" sheetId="9" r:id="R527ebc3b90bd441b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imaging" sheetId="10" r:id="Rcdc27f3595084e20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="11" r:id="R5b3a9b2dac3c4606"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="12" r:id="R70891447842a4584"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vitals" sheetId="13" r:id="R12a6fcded5784ddf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,7 +25,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="9">
+  <x:numFmts count="2">
+    <x:numFmt numFmtId="200" formatCode="0"/>
+    <x:numFmt numFmtId="201" formatCode="0.0"/>
+  </x:numFmts>
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -74,8 +79,13 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos Display"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF344054"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -102,8 +112,18 @@
         <x:fgColor rgb="FF1667A8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF123A63"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="16">
+  <x:borders count="17">
     <x:border/>
     <x:border>
       <x:left style="medium">
@@ -243,11 +263,25 @@
         <x:color rgb="FFC9D7E5"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD0D5DD"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD0D5DD"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD0D5DD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD0D5DD"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="108">
+  <x:cellXfs count="121">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -478,18 +512,81 @@
     <x:xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="9" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="9" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="1">
+  <x:dxfs count="5">
     <x:dxf>
       <x:font>
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE8F5E9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB42318"/>
+      </x:font>
+      <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE8F5E9"/>
+          <x:bgColor rgb="FFFEE4E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB42318"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFEE4E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB42318"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFEE4E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB42318"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFEE4E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -631,6 +728,31 @@
     <x:tableColumn id="12" name="RequestedBy"/>
     <x:tableColumn id="13" name="CreatedAt"/>
     <x:tableColumn id="14" name="CompletedAt"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="VitalsTable" displayName="VitalsTable" ref="A1:Q3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="17">
+    <x:tableColumn id="1" name="ExerciseId"/>
+    <x:tableColumn id="2" name="PatientId"/>
+    <x:tableColumn id="3" name="VitalId"/>
+    <x:tableColumn id="4" name="ExerciseMinute"/>
+    <x:tableColumn id="5" name="RecordedAt"/>
+    <x:tableColumn id="6" name="RecordedBy"/>
+    <x:tableColumn id="7" name="Source"/>
+    <x:tableColumn id="8" name="HeartRate"/>
+    <x:tableColumn id="9" name="SystolicBP"/>
+    <x:tableColumn id="10" name="DiastolicBP"/>
+    <x:tableColumn id="11" name="RespiratoryRate"/>
+    <x:tableColumn id="12" name="SpO2"/>
+    <x:tableColumn id="13" name="Temperature"/>
+    <x:tableColumn id="14" name="GCS"/>
+    <x:tableColumn id="15" name="BloodGlucose"/>
+    <x:tableColumn id="16" name="EtCO2"/>
+    <x:tableColumn id="17" name="PainScore"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -930,7 +1052,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B8" s="94" t="str">
-        <x:v>Lisa küsimused, analüüsid, uuringud ja tellimused vastavatele lehtedele.</x:v>
+        <x:v>Lisa elulised näitajad, küsimused, analüüsid, uuringud ja tellimused vastavatele lehtedele.</x:v>
       </x:c>
       <x:c r="C8" s="86"/>
       <x:c r="D8" s="95" t="str">
@@ -1085,9 +1207,17 @@
       <x:c r="A17" s="86"/>
       <x:c r="B17" s="86"/>
       <x:c r="C17" s="86"/>
-      <x:c r="D17" s="86"/>
-      <x:c r="E17" s="86"/>
-      <x:c r="F17" s="86"/>
+      <x:c r="D17" s="86" t="str">
+        <x:v>Vitals</x:v>
+      </x:c>
+      <x:c r="E17" s="86" t="n">
+        <x:f>SUMPRODUCT(--('Vitals'!A2:A200&lt;&gt;""))</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F17" s="86" t="str">
+        <x:f>IF(E17=0,"Tühi","Andmed olemas")</x:f>
+        <x:v>Andmed olemas</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="86"/>
@@ -1327,7 +1457,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R298121e0e16f4807"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c14b04f22fb4b80"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1599,7 +1729,218 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ed92dcf7677443d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c42fdc6c0af4bc7"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="10" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="14" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="9" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="16" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="11" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="113" t="str">
+        <x:v>ExerciseId</x:v>
+      </x:c>
+      <x:c r="B1" s="114" t="str">
+        <x:v>PatientId</x:v>
+      </x:c>
+      <x:c r="C1" s="114" t="str">
+        <x:v>VitalId</x:v>
+      </x:c>
+      <x:c r="D1" s="114" t="str">
+        <x:v>ExerciseMinute</x:v>
+      </x:c>
+      <x:c r="E1" s="114" t="str">
+        <x:v>RecordedAt</x:v>
+      </x:c>
+      <x:c r="F1" s="114" t="str">
+        <x:v>RecordedBy</x:v>
+      </x:c>
+      <x:c r="G1" s="114" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="H1" s="114" t="str">
+        <x:v>HeartRate</x:v>
+      </x:c>
+      <x:c r="I1" s="114" t="str">
+        <x:v>SystolicBP</x:v>
+      </x:c>
+      <x:c r="J1" s="114" t="str">
+        <x:v>DiastolicBP</x:v>
+      </x:c>
+      <x:c r="K1" s="114" t="str">
+        <x:v>RespiratoryRate</x:v>
+      </x:c>
+      <x:c r="L1" s="114" t="str">
+        <x:v>SpO2</x:v>
+      </x:c>
+      <x:c r="M1" s="114" t="str">
+        <x:v>Temperature</x:v>
+      </x:c>
+      <x:c r="N1" s="114" t="str">
+        <x:v>GCS</x:v>
+      </x:c>
+      <x:c r="O1" s="114" t="str">
+        <x:v>BloodGlucose</x:v>
+      </x:c>
+      <x:c r="P1" s="114" t="str">
+        <x:v>EtCO2</x:v>
+      </x:c>
+      <x:c r="Q1" s="115" t="str">
+        <x:v>PainScore</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="118" t="str">
+        <x:v>demo</x:v>
+      </x:c>
+      <x:c r="B2" s="118" t="str">
+        <x:v>PT-001</x:v>
+      </x:c>
+      <x:c r="C2" s="118" t="str">
+        <x:v>VITAL-001</x:v>
+      </x:c>
+      <x:c r="D2" s="119" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E2" s="118" t="str">
+        <x:v>09:22</x:v>
+      </x:c>
+      <x:c r="F2" s="118" t="str">
+        <x:v>EXCON</x:v>
+      </x:c>
+      <x:c r="G2" s="118" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="H2" s="119" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="I2" s="119" t="n">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="J2" s="119" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="K2" s="119" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="L2" s="119" t="n">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="M2" s="120" t="n">
+        <x:v>36.8</x:v>
+      </x:c>
+      <x:c r="N2" s="119" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="O2" s="120" t="n">
+        <x:v>6.1</x:v>
+      </x:c>
+      <x:c r="P2" s="120"/>
+      <x:c r="Q2" s="119" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="118" t="str">
+        <x:v>demo</x:v>
+      </x:c>
+      <x:c r="B3" s="118" t="str">
+        <x:v>PT-001</x:v>
+      </x:c>
+      <x:c r="C3" s="118" t="str">
+        <x:v>VITAL-002</x:v>
+      </x:c>
+      <x:c r="D3" s="119" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E3" s="118" t="str">
+        <x:v>09:32</x:v>
+      </x:c>
+      <x:c r="F3" s="118" t="str">
+        <x:v>EXCON</x:v>
+      </x:c>
+      <x:c r="G3" s="118" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="H3" s="119" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="I3" s="119" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="J3" s="119" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="K3" s="119" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="L3" s="119" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="M3" s="120" t="n">
+        <x:v>36.9</x:v>
+      </x:c>
+      <x:c r="N3" s="119" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="O3" s="120" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="P3" s="120"/>
+      <x:c r="Q3" s="119" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:conditionalFormatting sqref="H2:H200">
+    <x:cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
+      <x:formula>100</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="K2:K200">
+    <x:cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
+      <x:formula>20</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="L2:L200">
+    <x:cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
+      <x:formula>94</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="N2:N200">
+    <x:cfRule type="cellIs" dxfId="4" priority="4" operator="lessThan">
+      <x:formula>15</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="G2:G200">
+      <x:formula1>"scenario,manual"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ae0e58a232d40c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1709,7 +2050,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24a1fe3e78ed4ad3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae59a48248904dbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1804,7 +2145,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f04d8abb6024aeb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb819800df88144fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1892,7 +2233,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cd7c563aa9d4748"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14402807e30e44b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2040,7 +2381,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcac562182d96495b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76a8ee6bbd2b4732"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2220,7 +2561,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fd9f2366c8f45d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a2188d26ce1417e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2389,7 +2730,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30c3918294fd4360"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb00115d3325a40c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>